<commit_message>
feat(freemode): implementar flujo continuo por categoria seleccionada en Modo A la Carta
</commit_message>
<xml_diff>
--- a/assets/Dando Jugo Tarjetas.xlsx
+++ b/assets/Dando Jugo Tarjetas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\GitHub\Dando Jugo Web\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E38F89-9557-46C8-B2D8-48FB17335385}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FF3859-A394-4303-A702-3F702C8F645A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24945" windowHeight="8415" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24945" windowHeight="8415" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trivia" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Jugo" sheetId="3" r:id="rId3"/>
     <sheet name="Hoja 7" sheetId="4" r:id="rId4"/>
     <sheet name="Variables" sheetId="5" r:id="rId5"/>
-    <sheet name="Dando Jugo MiniJuegos" sheetId="6" r:id="rId6"/>
+    <sheet name="Otros Juegos" sheetId="6" r:id="rId6"/>
     <sheet name="Dando Jugo" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="791">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="777">
   <si>
     <t>ID</t>
   </si>
@@ -2125,39 +2125,12 @@
     <t>Apuestas si la siguiente carta es mayor o menor, cada 10 cartas, aumenta en 1 la cantidad de sorbos en juego</t>
   </si>
   <si>
-    <t>Piramide</t>
-  </si>
-  <si>
-    <t>Cada jugador tiene 2 cartas, por cada vez que salga la carta en la mano, debe realizar la acción de ese nivel (Tomar o regalar)</t>
-  </si>
-  <si>
-    <t>Veremos</t>
-  </si>
-  <si>
-    <t>Depende de encontrar una forma viable y limpia de mostrar el tablero</t>
-  </si>
-  <si>
     <t>Verdad o Reto</t>
   </si>
   <si>
     <t>Verdad o reto comun y corriente</t>
   </si>
   <si>
-    <t>Reloj</t>
-  </si>
-  <si>
-    <t>No se como explicarlo, pero el reloj</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Eliminado por convivencia</t>
-  </si>
-  <si>
     <t>Trivia Bomba</t>
   </si>
   <si>
@@ -2168,21 +2141,6 @@
   </si>
   <si>
     <t>Cambiar nombre</t>
-  </si>
-  <si>
-    <t>American Top Juice</t>
-  </si>
-  <si>
-    <t>Mimica, Karaoke, Descripción (Un hunt sin alternativas) (Se me ocurrio ahora). Sin equipos, con 2 jurado rotatorio y es el jurado quien adivina</t>
-  </si>
-  <si>
-    <t>No sé</t>
-  </si>
-  <si>
-    <t>Cambiado por charada</t>
-  </si>
-  <si>
-    <t>Juego de la moneda</t>
   </si>
   <si>
     <t>Charada</t>
@@ -18957,7 +18915,7 @@
         <v>442</v>
       </c>
       <c r="C56" s="37" t="s">
-        <v>776</v>
+        <v>762</v>
       </c>
       <c r="E56">
         <v>5</v>
@@ -18972,7 +18930,7 @@
         <v>442</v>
       </c>
       <c r="C57" s="37" t="s">
-        <v>777</v>
+        <v>763</v>
       </c>
       <c r="E57">
         <v>8</v>
@@ -22457,7 +22415,7 @@
         <v>501</v>
       </c>
       <c r="D2" s="36" t="s">
-        <v>717</v>
+        <v>703</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -22475,7 +22433,7 @@
         <v>503</v>
       </c>
       <c r="D3" s="36" t="s">
-        <v>718</v>
+        <v>704</v>
       </c>
       <c r="E3">
         <v>5</v>
@@ -22493,7 +22451,7 @@
         <v>505</v>
       </c>
       <c r="D4" s="36" t="s">
-        <v>719</v>
+        <v>705</v>
       </c>
       <c r="E4">
         <v>4</v>
@@ -22511,7 +22469,7 @@
         <v>507</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>720</v>
+        <v>706</v>
       </c>
       <c r="E5">
         <v>5</v>
@@ -22529,7 +22487,7 @@
         <v>509</v>
       </c>
       <c r="D6" s="36" t="s">
-        <v>721</v>
+        <v>707</v>
       </c>
       <c r="E6">
         <v>3</v>
@@ -22547,7 +22505,7 @@
         <v>511</v>
       </c>
       <c r="D7" s="36" t="s">
-        <v>722</v>
+        <v>708</v>
       </c>
       <c r="E7">
         <v>3</v>
@@ -22565,7 +22523,7 @@
         <v>513</v>
       </c>
       <c r="D8" s="36" t="s">
-        <v>723</v>
+        <v>709</v>
       </c>
       <c r="E8">
         <v>4</v>
@@ -22583,7 +22541,7 @@
         <v>515</v>
       </c>
       <c r="D9" s="36" t="s">
-        <v>724</v>
+        <v>710</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -22601,7 +22559,7 @@
         <v>517</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>725</v>
+        <v>711</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -22619,7 +22577,7 @@
         <v>519</v>
       </c>
       <c r="D11" s="36" t="s">
-        <v>726</v>
+        <v>712</v>
       </c>
       <c r="E11">
         <v>7</v>
@@ -22637,7 +22595,7 @@
         <v>521</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>727</v>
+        <v>713</v>
       </c>
       <c r="E12">
         <v>4</v>
@@ -22655,7 +22613,7 @@
         <v>523</v>
       </c>
       <c r="D13" s="36" t="s">
-        <v>728</v>
+        <v>714</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -22673,7 +22631,7 @@
         <v>525</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>729</v>
+        <v>715</v>
       </c>
       <c r="E14">
         <v>8</v>
@@ -22691,7 +22649,7 @@
         <v>527</v>
       </c>
       <c r="D15" s="36" t="s">
-        <v>730</v>
+        <v>716</v>
       </c>
       <c r="E15">
         <v>6</v>
@@ -22709,7 +22667,7 @@
         <v>529</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>731</v>
+        <v>717</v>
       </c>
       <c r="E16">
         <v>8</v>
@@ -22727,7 +22685,7 @@
         <v>531</v>
       </c>
       <c r="D17" s="36" t="s">
-        <v>732</v>
+        <v>718</v>
       </c>
       <c r="E17">
         <v>7</v>
@@ -22745,7 +22703,7 @@
         <v>533</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>733</v>
+        <v>719</v>
       </c>
       <c r="E18">
         <v>6</v>
@@ -22763,7 +22721,7 @@
         <v>535</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>734</v>
+        <v>720</v>
       </c>
       <c r="E19">
         <v>7</v>
@@ -22781,7 +22739,7 @@
         <v>537</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>735</v>
+        <v>721</v>
       </c>
       <c r="E20">
         <v>7</v>
@@ -22799,7 +22757,7 @@
         <v>539</v>
       </c>
       <c r="D21" s="36" t="s">
-        <v>736</v>
+        <v>722</v>
       </c>
       <c r="E21">
         <v>5</v>
@@ -22817,7 +22775,7 @@
         <v>541</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>737</v>
+        <v>723</v>
       </c>
       <c r="E22">
         <v>5</v>
@@ -22835,7 +22793,7 @@
         <v>543</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>738</v>
+        <v>724</v>
       </c>
       <c r="E23">
         <v>4</v>
@@ -22853,7 +22811,7 @@
         <v>545</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>739</v>
+        <v>725</v>
       </c>
       <c r="E24">
         <v>6</v>
@@ -22871,7 +22829,7 @@
         <v>547</v>
       </c>
       <c r="D25" s="36" t="s">
-        <v>740</v>
+        <v>726</v>
       </c>
       <c r="E25">
         <v>4</v>
@@ -22889,7 +22847,7 @@
         <v>549</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>741</v>
+        <v>727</v>
       </c>
       <c r="E26">
         <v>2</v>
@@ -22907,7 +22865,7 @@
         <v>551</v>
       </c>
       <c r="D27" s="36" t="s">
-        <v>742</v>
+        <v>728</v>
       </c>
       <c r="E27">
         <v>2</v>
@@ -22925,7 +22883,7 @@
         <v>553</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>743</v>
+        <v>729</v>
       </c>
       <c r="E28">
         <v>2</v>
@@ -22943,7 +22901,7 @@
         <v>555</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>744</v>
+        <v>730</v>
       </c>
       <c r="E29">
         <v>8</v>
@@ -22961,7 +22919,7 @@
         <v>557</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>745</v>
+        <v>731</v>
       </c>
       <c r="E30">
         <v>4</v>
@@ -22979,7 +22937,7 @@
         <v>559</v>
       </c>
       <c r="D31" s="36" t="s">
-        <v>746</v>
+        <v>732</v>
       </c>
       <c r="E31">
         <v>5</v>
@@ -22997,7 +22955,7 @@
         <v>561</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>747</v>
+        <v>733</v>
       </c>
       <c r="E32">
         <v>3</v>
@@ -23015,7 +22973,7 @@
         <v>563</v>
       </c>
       <c r="D33" s="36" t="s">
-        <v>748</v>
+        <v>734</v>
       </c>
       <c r="E33">
         <v>8</v>
@@ -23033,7 +22991,7 @@
         <v>565</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>749</v>
+        <v>735</v>
       </c>
       <c r="E34">
         <v>6</v>
@@ -23051,7 +23009,7 @@
         <v>567</v>
       </c>
       <c r="D35" s="36" t="s">
-        <v>750</v>
+        <v>736</v>
       </c>
       <c r="E35">
         <v>4</v>
@@ -23069,7 +23027,7 @@
         <v>569</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>751</v>
+        <v>737</v>
       </c>
       <c r="E36">
         <v>5</v>
@@ -23087,7 +23045,7 @@
         <v>571</v>
       </c>
       <c r="D37" s="36" t="s">
-        <v>752</v>
+        <v>738</v>
       </c>
       <c r="E37">
         <v>3</v>
@@ -23105,7 +23063,7 @@
         <v>573</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>753</v>
+        <v>739</v>
       </c>
       <c r="E38">
         <v>6</v>
@@ -23123,7 +23081,7 @@
         <v>575</v>
       </c>
       <c r="D39" s="36" t="s">
-        <v>754</v>
+        <v>740</v>
       </c>
       <c r="E39">
         <v>2</v>
@@ -23141,7 +23099,7 @@
         <v>577</v>
       </c>
       <c r="D40" s="36" t="s">
-        <v>755</v>
+        <v>741</v>
       </c>
       <c r="E40">
         <v>9</v>
@@ -23159,7 +23117,7 @@
         <v>579</v>
       </c>
       <c r="D41" s="36" t="s">
-        <v>756</v>
+        <v>742</v>
       </c>
       <c r="E41">
         <v>6</v>
@@ -26478,7 +26436,7 @@
         <v>634</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>757</v>
+        <v>743</v>
       </c>
       <c r="G22" s="10" t="s">
         <v>18</v>
@@ -26495,7 +26453,7 @@
         <v>635</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>758</v>
+        <v>744</v>
       </c>
       <c r="G23" s="10" t="s">
         <v>18</v>
@@ -26512,7 +26470,7 @@
         <v>637</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>759</v>
+        <v>745</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -26529,7 +26487,7 @@
         <v>639</v>
       </c>
       <c r="D25" s="36" t="s">
-        <v>760</v>
+        <v>746</v>
       </c>
       <c r="G25" s="10" t="s">
         <v>18</v>
@@ -26546,7 +26504,7 @@
         <v>641</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>761</v>
+        <v>747</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -26563,7 +26521,7 @@
         <v>643</v>
       </c>
       <c r="D27" s="36" t="s">
-        <v>762</v>
+        <v>748</v>
       </c>
       <c r="G27" s="10" t="s">
         <v>18</v>
@@ -26580,7 +26538,7 @@
         <v>645</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>763</v>
+        <v>749</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>18</v>
@@ -26597,7 +26555,7 @@
         <v>647</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>764</v>
+        <v>750</v>
       </c>
       <c r="G29" s="10" t="s">
         <v>18</v>
@@ -26614,7 +26572,7 @@
         <v>649</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>765</v>
+        <v>751</v>
       </c>
       <c r="G30" s="10" t="s">
         <v>18</v>
@@ -26631,7 +26589,7 @@
         <v>651</v>
       </c>
       <c r="D31" s="36" t="s">
-        <v>766</v>
+        <v>752</v>
       </c>
       <c r="G31" s="10" t="s">
         <v>18</v>
@@ -26648,7 +26606,7 @@
         <v>653</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>767</v>
+        <v>753</v>
       </c>
       <c r="G32" s="10" t="s">
         <v>18</v>
@@ -26665,7 +26623,7 @@
         <v>655</v>
       </c>
       <c r="D33" s="36" t="s">
-        <v>768</v>
+        <v>754</v>
       </c>
       <c r="G33" s="10" t="s">
         <v>18</v>
@@ -26682,7 +26640,7 @@
         <v>657</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>769</v>
+        <v>755</v>
       </c>
       <c r="G34" s="25"/>
     </row>
@@ -26697,7 +26655,7 @@
         <v>659</v>
       </c>
       <c r="D35" s="36" t="s">
-        <v>770</v>
+        <v>756</v>
       </c>
       <c r="G35" s="25"/>
     </row>
@@ -26712,7 +26670,7 @@
         <v>661</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>771</v>
+        <v>757</v>
       </c>
       <c r="G36" s="25"/>
     </row>
@@ -26727,7 +26685,7 @@
         <v>663</v>
       </c>
       <c r="D37" s="36" t="s">
-        <v>772</v>
+        <v>758</v>
       </c>
       <c r="G37" s="25"/>
     </row>
@@ -26742,7 +26700,7 @@
         <v>665</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>773</v>
+        <v>759</v>
       </c>
       <c r="G38" s="25"/>
     </row>
@@ -26757,7 +26715,7 @@
         <v>667</v>
       </c>
       <c r="D39" s="36" t="s">
-        <v>774</v>
+        <v>760</v>
       </c>
       <c r="G39" s="25"/>
     </row>
@@ -26772,7 +26730,7 @@
         <v>668</v>
       </c>
       <c r="D40" s="36" t="s">
-        <v>758</v>
+        <v>744</v>
       </c>
       <c r="G40" s="25"/>
     </row>
@@ -26787,7 +26745,7 @@
         <v>670</v>
       </c>
       <c r="D41" s="36" t="s">
-        <v>775</v>
+        <v>761</v>
       </c>
       <c r="G41" s="25"/>
     </row>
@@ -29744,7 +29702,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G999"/>
+  <dimension ref="A1:G995"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
@@ -29857,7 +29815,7 @@
       <c r="A6" s="33" t="s">
         <v>696</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="33" t="s">
         <v>697</v>
       </c>
       <c r="C6" s="33">
@@ -29865,123 +29823,78 @@
       </c>
       <c r="D6" s="35"/>
       <c r="E6" s="33" t="s">
-        <v>698</v>
+        <v>18</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>698</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>699</v>
+        <v>687</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
-        <v>700</v>
-      </c>
-      <c r="B7" s="33" t="s">
-        <v>701</v>
+        <v>698</v>
+      </c>
+      <c r="B7" s="34" t="s">
+        <v>699</v>
       </c>
       <c r="C7" s="33">
         <v>2</v>
       </c>
       <c r="D7" s="35"/>
       <c r="E7" s="33" t="s">
-        <v>18</v>
+        <v>700</v>
       </c>
       <c r="F7" s="33" t="s">
         <v>687</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>701</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
         <v>702</v>
       </c>
-      <c r="B8" s="33" t="s">
-        <v>703</v>
-      </c>
-      <c r="C8" s="33">
-        <v>2</v>
-      </c>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
       <c r="D8" s="35"/>
       <c r="E8" s="33" t="s">
-        <v>704</v>
+        <v>700</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>705</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="33" t="s">
-        <v>707</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>708</v>
-      </c>
-      <c r="C9" s="33">
-        <v>2</v>
-      </c>
+      <c r="A9" s="35"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
       <c r="D9" s="35"/>
-      <c r="E9" s="33" t="s">
-        <v>709</v>
-      </c>
-      <c r="F9" s="33" t="s">
-        <v>687</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>710</v>
-      </c>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>711</v>
-      </c>
-      <c r="B10" s="32" t="s">
-        <v>712</v>
-      </c>
-      <c r="C10" s="33">
-        <v>3</v>
-      </c>
+      <c r="A10" s="35"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
       <c r="D10" s="35"/>
-      <c r="E10" s="33" t="s">
-        <v>704</v>
-      </c>
-      <c r="F10" s="33" t="s">
-        <v>713</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>714</v>
-      </c>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="33" t="s">
-        <v>715</v>
-      </c>
-      <c r="B11" s="33"/>
+      <c r="A11" s="35"/>
+      <c r="B11" s="35"/>
       <c r="C11" s="35"/>
       <c r="D11" s="35"/>
-      <c r="E11" s="33" t="s">
-        <v>709</v>
-      </c>
-      <c r="F11" s="33" t="s">
-        <v>687</v>
-      </c>
+      <c r="E11" s="35"/>
+      <c r="F11" s="35"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="33" t="s">
-        <v>716</v>
-      </c>
+      <c r="A12" s="35"/>
       <c r="B12" s="35"/>
       <c r="C12" s="35"/>
       <c r="D12" s="35"/>
-      <c r="E12" s="33" t="s">
-        <v>709</v>
-      </c>
-      <c r="F12" s="33" t="s">
-        <v>709</v>
-      </c>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="35"/>
@@ -37846,38 +37759,6 @@
       <c r="D995" s="35"/>
       <c r="E995" s="35"/>
       <c r="F995" s="35"/>
-    </row>
-    <row r="996" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A996" s="35"/>
-      <c r="B996" s="35"/>
-      <c r="C996" s="35"/>
-      <c r="D996" s="35"/>
-      <c r="E996" s="35"/>
-      <c r="F996" s="35"/>
-    </row>
-    <row r="997" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A997" s="35"/>
-      <c r="B997" s="35"/>
-      <c r="C997" s="35"/>
-      <c r="D997" s="35"/>
-      <c r="E997" s="35"/>
-      <c r="F997" s="35"/>
-    </row>
-    <row r="998" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A998" s="35"/>
-      <c r="B998" s="35"/>
-      <c r="C998" s="35"/>
-      <c r="D998" s="35"/>
-      <c r="E998" s="35"/>
-      <c r="F998" s="35"/>
-    </row>
-    <row r="999" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A999" s="35"/>
-      <c r="B999" s="35"/>
-      <c r="C999" s="35"/>
-      <c r="D999" s="35"/>
-      <c r="E999" s="35"/>
-      <c r="F999" s="35"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -37904,51 +37785,51 @@
         <v>679</v>
       </c>
       <c r="C1" s="38" t="s">
-        <v>778</v>
+        <v>764</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="37" t="s">
-        <v>779</v>
+        <v>765</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>783</v>
+        <v>769</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>784</v>
+        <v>770</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="37" t="s">
-        <v>782</v>
+        <v>768</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>785</v>
+        <v>771</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>786</v>
+        <v>772</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="37" t="s">
-        <v>781</v>
+        <v>767</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>787</v>
+        <v>773</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>788</v>
+        <v>774</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="s">
-        <v>780</v>
+        <v>766</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>789</v>
+        <v>775</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>790</v>
+        <v>776</v>
       </c>
     </row>
   </sheetData>

</xml_diff>